<commit_message>
members S15 indicator in one student's name
</commit_message>
<xml_diff>
--- a/S15/_members_s15.xlsx
+++ b/S15/_members_s15.xlsx
@@ -70,7 +70,7 @@
     <t xml:space="preserve">999796</t>
   </si>
   <si>
-    <t xml:space="preserve">Ville Nylander</t>
+    <t xml:space="preserve">Ville Nylander 1</t>
   </si>
   <si>
     <t xml:space="preserve">635821</t>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="G74" s="1" t="n">
         <f aca="true">RAND()</f>
-        <v>0.0520562998062195</v>
+        <v>0.740398563174401</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>